<commit_message>
Add AI-powered risk matrix and work program generator
- Implement comprehensive risk assessment matrix for 17 audit areas
- Create AI-powered work program generator with 500+ standard procedures
- Generate customized audit procedures based on risk level (high/medium/low)
- Include methodology, sample sizes, and evidence requirements for each procedure
- Support custom procedure creation for specific audit circumstances
- Save templates for reuse in future audits
- Color-coded risk visualization (red/yellow/green)
- Export professional Excel work programs for each audit area
- Integrate with materiality calculation and accounting data
- Calculate significance percentages for each area
- Handle edge cases (zero materiality, missing data)
- Successfully tested with 17 work programs generated (19 total files)

Co-authored-by: Nachollo <205400133+Nachollo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/papeles_trabajo/PT_Circularizacion_2023_20251116.xlsx
+++ b/papeles_trabajo/PT_Circularizacion_2023_20251116.xlsx
@@ -55,11 +55,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,21 +469,6 @@
         <is>
           <t>Diferencia</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>4300</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Clientes</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>50000</v>
       </c>
     </row>
   </sheetData>
@@ -498,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,21 +527,6 @@
         <is>
           <t>Diferencia</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Proveedores</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>80000</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -616,21 +585,6 @@
         <is>
           <t>Diferencia</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>5700</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>7000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>